<commit_message>
read data and add to queue
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\UiPath\IJ_WysylanieFaktur\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FAE9DC7-F895-4955-9136-6DF1C2A4ACBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5991767-CE53-4180-AE9F-23A1E9D6BE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="51">
   <si>
     <t>Name</t>
   </si>
@@ -133,6 +133,48 @@
   </si>
   <si>
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
+  </si>
+  <si>
+    <t>WorkbookAddress</t>
+  </si>
+  <si>
+    <t>SheetName</t>
+  </si>
+  <si>
+    <t>C:\Users\Administrator\Downloads\EWIDENCJA I ROZLICZENIE - GRUDZIEŃ 2025.xlsx</t>
+  </si>
+  <si>
+    <t>PLACÓWKI ROZLICZENIE</t>
+  </si>
+  <si>
+    <t>Range</t>
+  </si>
+  <si>
+    <t>I:N</t>
+  </si>
+  <si>
+    <t>DANE DO FAKTURY</t>
+  </si>
+  <si>
+    <t>ColumnData</t>
+  </si>
+  <si>
+    <t>NIPRegex</t>
+  </si>
+  <si>
+    <t>\d[\d| |-]{7,13}\d</t>
+  </si>
+  <si>
+    <t>ColumnKwota</t>
+  </si>
+  <si>
+    <t>KWOTA DO FAKTURY</t>
+  </si>
+  <si>
+    <t>ColumnNumerFaktury</t>
+  </si>
+  <si>
+    <t>NUMER FAKTURY</t>
   </si>
 </sst>
 </file>
@@ -541,13 +583,62 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="2" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+    </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>